<commit_message>
update schedule for 2026 term with new topics and dates
</commit_message>
<xml_diff>
--- a/syllabus/AREC 615 Class Schedule.xlsx
+++ b/syllabus/AREC 615 Class Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/judebayham/Documents/git_projects/arec-615/syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8337A5-AB5F-8F43-B400-A8DB2DAAB436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E3603DD-4C2E-1E4B-B0EA-09DD42391A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36840" yWindow="1120" windowWidth="34560" windowHeight="20320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FA2025" sheetId="6" r:id="rId1"/>
@@ -74,38 +74,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
-  <si>
-    <t>LP Solution - Simplex Method</t>
-  </si>
-  <si>
-    <t>LP Sensitivity</t>
-  </si>
-  <si>
-    <t>LP Duality</t>
-  </si>
-  <si>
-    <t>Unconstrained nonlinear optimization</t>
-  </si>
-  <si>
-    <t>Constrained nonlinear optimization</t>
-  </si>
-  <si>
-    <t>Constrained nonlinear optimization: numerical methods</t>
-  </si>
-  <si>
-    <t>Regression applications: likelihood estimation</t>
-  </si>
-  <si>
-    <t>Regression applications: generalized method of moments</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
     <t>Review</t>
   </si>
   <si>
-    <t>Exam 1</t>
-  </si>
-  <si>
     <t>Value function iteration and policy iteration using approximation</t>
   </si>
   <si>
@@ -130,109 +103,58 @@
     <t>due</t>
   </si>
   <si>
-    <t>Problem Set 1</t>
-  </si>
-  <si>
-    <t>Problem Set 2</t>
-  </si>
-  <si>
-    <t>Problem Set 3</t>
-  </si>
-  <si>
-    <t>Problem Set 4</t>
-  </si>
-  <si>
-    <t>M&amp;S 1</t>
-  </si>
-  <si>
-    <t>M&amp;S 2-3</t>
-  </si>
-  <si>
-    <t>M&amp;S 3</t>
-  </si>
-  <si>
-    <t>M&amp;S 7</t>
-  </si>
-  <si>
-    <t>M&amp;F 3</t>
-  </si>
-  <si>
-    <t>M&amp;S 12</t>
-  </si>
-  <si>
-    <t>M&amp;F 7</t>
-  </si>
-  <si>
-    <t>M&amp;F 8</t>
-  </si>
-  <si>
-    <t>M&amp;F 9</t>
-  </si>
-  <si>
-    <t>Input-Output Modeling</t>
-  </si>
-  <si>
-    <t>Intro &amp; Start Linear Programming</t>
-  </si>
-  <si>
-    <t>Numerical Foundations</t>
-  </si>
-  <si>
-    <t>No Class</t>
-  </si>
-  <si>
-    <t>Foundations of dynamic programming</t>
-  </si>
-  <si>
-    <t>Discrete-state DP with finite horizon</t>
-  </si>
-  <si>
-    <t>Infinite-horizon DP</t>
-  </si>
-  <si>
-    <t>Functional equations and value function properties</t>
-  </si>
-  <si>
-    <t>Dynamic models with continuous state</t>
-  </si>
-  <si>
-    <t>Value and policy functions in continuous spaces</t>
-  </si>
-  <si>
-    <t>Collocation and projection methods</t>
-  </si>
-  <si>
     <t>Potential topics</t>
   </si>
   <si>
-    <t>Final Exam (Wednesday 6:20 - 8:20 PM)</t>
-  </si>
-  <si>
-    <t>How to present</t>
-  </si>
-  <si>
-    <t>Select Project Paper</t>
-  </si>
-  <si>
-    <t>Replication and Extension Proposal</t>
-  </si>
-  <si>
-    <t>Fenichel Abbott - Metaphor to measurement</t>
-  </si>
-  <si>
-    <t>Burt - Optimal Resource Use</t>
-  </si>
-  <si>
-    <t>Project workshop</t>
-  </si>
-  <si>
-    <t>Presentation: Shuhang, Catherine, Shreezal</t>
-  </si>
-  <si>
-    <t>Presentation: Alisha, Suchil, Matt</t>
-  </si>
-  <si>
-    <t>Presentation: Jayna, Trent, Mehran</t>
+    <t>Course orientation; R and AI setup</t>
+  </si>
+  <si>
+    <t>Math/R refresh</t>
+  </si>
+  <si>
+    <t>Linear Programming: formulation and graphical interpretation</t>
+  </si>
+  <si>
+    <t>LP formulation from data</t>
+  </si>
+  <si>
+    <t>Applied LP: solving and interpreting a model</t>
+  </si>
+  <si>
+    <t>LP sensitivity and shadow values</t>
+  </si>
+  <si>
+    <t>LP duality as economic interpretation</t>
+  </si>
+  <si>
+    <t>Presentation/discussion</t>
+  </si>
+  <si>
+    <t>Midterm 1</t>
+  </si>
+  <si>
+    <t>Karush Kuhn Tucker and corner solutions</t>
+  </si>
+  <si>
+    <t>Midterm 2</t>
+  </si>
+  <si>
+    <t>Unconstrained and constrained nonlinear optimization + Numerical foundations: roots, diagnostics, and convergence</t>
+  </si>
+  <si>
+    <t>Risk, uncertainty, and scenario analysis in static models</t>
+  </si>
+  <si>
+    <t>Finite-horizon dynamic programming and backward induction</t>
+  </si>
+  <si>
+    <t>Infinite-horizon Bellman equation and value function iteration</t>
+  </si>
+  <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>Flex Day</t>
   </si>
 </sst>
 </file>
@@ -260,7 +182,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,20 +191,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4A86E8"/>
-        <bgColor rgb="FF4A86E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -298,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -307,25 +217,30 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -665,50 +580,46 @@
   <sheetData>
     <row r="1" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="14" x14ac:dyDescent="0.15">
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="5">
-        <v>45895</v>
+      <c r="B2" s="4">
+        <v>46259</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>22</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
     <row r="3" spans="1:5" ht="14" x14ac:dyDescent="0.15">
       <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="4">
         <f t="shared" ref="B3" si="0">B2+2</f>
-        <v>45897</v>
+        <v>46261</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>23</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" ht="14" x14ac:dyDescent="0.15">
@@ -716,112 +627,102 @@
         <f t="shared" ref="A4:A33" si="1">A2+1</f>
         <v>2</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="4">
         <f>B2+7</f>
-        <v>45902</v>
+        <v>46266</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>24</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A5" s="2">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="4">
         <f t="shared" ref="B5" si="2">B4+2</f>
-        <v>45904</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>2</v>
+        <v>46268</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>13</v>
       </c>
       <c r="D5" s="3"/>
     </row>
-    <row r="6" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A6" s="2">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="4">
         <f>B4+7</f>
-        <v>45909</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>25</v>
-      </c>
+        <v>46273</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A7" s="2">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="4">
         <f t="shared" ref="B7" si="3">B6+2</f>
-        <v>45911</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+        <v>46275</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="3"/>
+    </row>
+    <row r="8" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A8" s="2">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <f>B6+7</f>
-        <v>45916</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+        <v>46280</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="7"/>
+    </row>
+    <row r="9" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="2">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="4">
         <f t="shared" ref="B9" si="4">B8+2</f>
-        <v>45918</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>6</v>
+        <v>46282</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A10" s="2">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="B10" s="9">
         <f>B8+7</f>
-        <v>45923</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="7"/>
+        <v>46287</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="6"/>
       <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:5" ht="14" x14ac:dyDescent="0.15">
@@ -829,129 +730,125 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <f t="shared" ref="B11" si="5">B10+2</f>
-        <v>45925</v>
+        <v>46289</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A12" s="2">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <f>B10+7</f>
-        <v>45930</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>5</v>
+        <v>46294</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="D12" s="3"/>
     </row>
-    <row r="13" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="2">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="4">
         <f t="shared" ref="B13" si="6">B12+2</f>
-        <v>45932</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="10" t="s">
-        <v>45</v>
-      </c>
+        <v>46296</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="2">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="4">
         <f>B12+7</f>
-        <v>45937</v>
-      </c>
-      <c r="D14" s="8"/>
+        <v>46301</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="7"/>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="2">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="4">
         <f t="shared" ref="B15" si="7">B14+2</f>
-        <v>45939</v>
-      </c>
-      <c r="C15" s="3" t="s">
+        <v>46303</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="7"/>
+    </row>
+    <row r="16" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A16" s="2">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="E15" s="8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A16" s="2">
+      <c r="B16" s="4">
+        <f>B14+7</f>
+        <v>46308</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="3"/>
+    </row>
+    <row r="17" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A17" s="2">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="B16" s="5">
-        <f>B14+7</f>
-        <v>45944</v>
-      </c>
-      <c r="C16" s="3" t="s">
+      <c r="B17" s="4">
+        <f t="shared" ref="B17" si="8">B16+2</f>
+        <v>46310</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A18" s="2">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="D16" s="3"/>
-    </row>
-    <row r="17" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A17" s="2">
-        <f t="shared" si="1"/>
-        <v>8</v>
-      </c>
-      <c r="B17" s="5">
-        <f t="shared" ref="B17" si="8">B16+2</f>
-        <v>45946</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A18" s="2">
+      <c r="B18" s="4">
+        <f>B16+7</f>
+        <v>46315</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+      <c r="A19" s="2">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="B18" s="5">
-        <f>B16+7</f>
-        <v>45951</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A19" s="2">
-        <f t="shared" si="1"/>
-        <v>9</v>
-      </c>
-      <c r="B19" s="5">
+      <c r="B19" s="4">
         <f t="shared" ref="B19" si="9">B18+2</f>
-        <v>45953</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>37</v>
+        <v>46317</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="14" x14ac:dyDescent="0.15">
@@ -959,78 +856,70 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="4">
         <f>B18+7</f>
-        <v>45958</v>
+        <v>46322</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A21" s="2">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="4">
         <f t="shared" ref="B21" si="10">B20+2</f>
-        <v>45960</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+        <v>46324</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="3"/>
+      <c r="E21" s="7"/>
+    </row>
+    <row r="22" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A22" s="2">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="B22" s="5">
+      <c r="B22" s="4">
         <f>B20+7</f>
-        <v>45965</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>40</v>
+        <v>46329</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D22" s="3"/>
-      <c r="E22" s="8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+      <c r="E22" s="7"/>
+    </row>
+    <row r="23" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A23" s="2">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="B23" s="5">
+      <c r="B23" s="4">
         <f t="shared" ref="B23" si="11">B22+2</f>
-        <v>45967</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+        <v>46331</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="3"/>
+    </row>
+    <row r="24" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A24" s="2">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="B24" s="5">
+      <c r="B24" s="4">
         <f>B22+7</f>
-        <v>45972</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>47</v>
+        <v>46336</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="14" x14ac:dyDescent="0.15">
@@ -1038,12 +927,12 @@
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="B25" s="5">
+      <c r="B25" s="4">
         <f t="shared" ref="B25" si="12">B24+2</f>
-        <v>45974</v>
+        <v>46338</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="D25" s="3"/>
     </row>
@@ -1052,133 +941,80 @@
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="B26" s="5">
+      <c r="B26" s="4">
         <f>B24+7</f>
-        <v>45979</v>
+        <v>46343</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="D26" s="3"/>
-      <c r="E26" s="8" t="s">
-        <v>21</v>
-      </c>
+      <c r="E26" s="7"/>
     </row>
     <row r="27" spans="1:5" ht="14" x14ac:dyDescent="0.15">
       <c r="A27" s="2">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="B27" s="5">
+      <c r="B27" s="4">
         <f t="shared" ref="B27" si="13">B26+2</f>
-        <v>45981</v>
+        <v>46345</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A28" s="2">
-        <f t="shared" si="1"/>
-        <v>14</v>
-      </c>
-      <c r="B28" s="5">
-        <f>B26+7</f>
-        <v>45986</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A29" s="2">
-        <f t="shared" si="1"/>
-        <v>14</v>
-      </c>
-      <c r="B29" s="5">
-        <f t="shared" ref="B29" si="14">B28+2</f>
-        <v>45988</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A30" s="2">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="B30" s="5">
-        <f>B28+7</f>
-        <v>45993</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>50</v>
-      </c>
+    <row r="28" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A28" s="10"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="11"/>
+    </row>
+    <row r="29" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A29" s="10"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="11"/>
+    </row>
+    <row r="30" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A30" s="10"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="11"/>
       <c r="D30" s="3"/>
     </row>
-    <row r="31" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A31" s="2">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="B31" s="5">
-        <f t="shared" ref="B31" si="15">B30+2</f>
-        <v>45995</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>51</v>
-      </c>
+    <row r="31" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A31" s="10"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="11"/>
       <c r="D31" s="1"/>
       <c r="E31" s="3"/>
     </row>
     <row r="32" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A32" s="2">
-        <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="B32" s="5">
-        <f>B30+7</f>
-        <v>46000</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>52</v>
-      </c>
+      <c r="A32" s="10"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="12"/>
     </row>
     <row r="33" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A33" s="2">
-        <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="B33" s="5">
-        <f t="shared" ref="B33" si="16">B32+2</f>
-        <v>46002</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A33" s="10"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="12"/>
     </row>
     <row r="34" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="B34" s="5">
-        <v>46008</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>43</v>
-      </c>
+      <c r="A34" s="13"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="12"/>
     </row>
     <row r="35" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="B35" s="5"/>
-      <c r="C35" s="8"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="7"/>
     </row>
     <row r="36" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="B36" s="5"/>
+      <c r="B36" s="4"/>
       <c r="C36" s="3"/>
-      <c r="D36" s="6"/>
+      <c r="D36" s="5"/>
     </row>
     <row r="37" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="B37" s="5"/>
+      <c r="B37" s="4"/>
       <c r="C37" s="1"/>
       <c r="D37" s="3"/>
     </row>
@@ -1187,16 +1023,16 @@
     </row>
     <row r="39" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="C39" s="1"/>
-      <c r="D39" s="8"/>
+      <c r="D39" s="7"/>
     </row>
     <row r="40" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="C40" s="1"/>
+      <c r="C40" s="7"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
     </row>
     <row r="41" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="C41" s="1"/>
-      <c r="D41" s="8"/>
+      <c r="D41" s="7"/>
     </row>
     <row r="42" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="C42" s="1"/>
@@ -2162,23 +1998,23 @@
   </cols>
   <sheetData>
     <row r="15" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A15" s="8" t="s">
-        <v>42</v>
+      <c r="A15" s="7" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="14" x14ac:dyDescent="0.15">
-      <c r="B16" s="10" t="s">
-        <v>10</v>
+      <c r="B16" s="8" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="2:2" ht="14" x14ac:dyDescent="0.15">
       <c r="B17" s="3" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="2:2" ht="14" x14ac:dyDescent="0.15">
       <c r="B18" s="3" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update course materials; enhance schedule, modify notes, and adjust presentation styles
</commit_message>
<xml_diff>
--- a/syllabus/AREC 615 Class Schedule.xlsx
+++ b/syllabus/AREC 615 Class Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/judebayham/Documents/git_projects/arec-615/syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E3603DD-4C2E-1E4B-B0EA-09DD42391A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6120A27-3ED7-114A-BC82-C6F4B36C8A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-36840" yWindow="1120" windowWidth="34560" windowHeight="20320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
   <si>
     <t>Review</t>
   </si>
@@ -109,18 +109,12 @@
     <t>Course orientation; R and AI setup</t>
   </si>
   <si>
-    <t>Math/R refresh</t>
-  </si>
-  <si>
     <t>Linear Programming: formulation and graphical interpretation</t>
   </si>
   <si>
     <t>LP formulation from data</t>
   </si>
   <si>
-    <t>Applied LP: solving and interpreting a model</t>
-  </si>
-  <si>
     <t>LP sensitivity and shadow values</t>
   </si>
   <si>
@@ -155,6 +149,18 @@
   </si>
   <si>
     <t>Flex Day</t>
+  </si>
+  <si>
+    <t>Stewart &amp; Greenhalgh (1977)</t>
+  </si>
+  <si>
+    <t>LP Application</t>
+  </si>
+  <si>
+    <t>LP: solving and interpreting a model</t>
+  </si>
+  <si>
+    <t>McCarl &amp; Spreen Chapter 1</t>
   </si>
 </sst>
 </file>
@@ -605,7 +611,9 @@
       <c r="C2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3"/>
+      <c r="D2" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="E2" s="3"/>
     </row>
     <row r="3" spans="1:5" ht="14" x14ac:dyDescent="0.15">
@@ -622,7 +630,7 @@
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A4" s="2">
         <f t="shared" ref="A4:A33" si="1">A2+1</f>
         <v>2</v>
@@ -631,7 +639,7 @@
         <f>B2+7</f>
         <v>46266</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="3"/>
@@ -647,7 +655,7 @@
         <v>46268</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="D5" s="3"/>
     </row>
@@ -661,12 +669,12 @@
         <v>46273</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:5" ht="14" x14ac:dyDescent="0.15">
       <c r="A7" s="2">
         <f t="shared" si="1"/>
         <v>3</v>
@@ -676,9 +684,11 @@
         <v>46275</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="3"/>
+        <v>26</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A8" s="2">
@@ -690,7 +700,7 @@
         <v>46280</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="7"/>
@@ -705,7 +715,7 @@
         <v>46282</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -720,7 +730,7 @@
         <v>46287</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="3"/>
@@ -748,7 +758,7 @@
         <v>46294</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D12" s="3"/>
     </row>
@@ -762,7 +772,7 @@
         <v>46296</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="8"/>
@@ -777,7 +787,7 @@
         <v>46301</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D14" s="7"/>
       <c r="E14" s="3"/>
@@ -792,7 +802,7 @@
         <v>46303</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E15" s="7"/>
     </row>
@@ -806,7 +816,7 @@
         <v>46308</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D16" s="3"/>
     </row>
@@ -820,7 +830,7 @@
         <v>46310</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E17" s="3"/>
     </row>
@@ -834,7 +844,7 @@
         <v>46315</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D18" s="3"/>
     </row>
@@ -861,7 +871,7 @@
         <v>46322</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E20" s="3"/>
     </row>
@@ -875,7 +885,7 @@
         <v>46324</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="7"/>
@@ -890,7 +900,7 @@
         <v>46329</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="7"/>
@@ -905,7 +915,7 @@
         <v>46331</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D23" s="3"/>
     </row>
@@ -919,7 +929,7 @@
         <v>46336</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="14" x14ac:dyDescent="0.15">
@@ -932,7 +942,7 @@
         <v>46338</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D25" s="3"/>
     </row>
@@ -961,7 +971,7 @@
         <v>46345</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>

</xml_diff>

<commit_message>
Update course schedule with revised topics and readings for clarity
</commit_message>
<xml_diff>
--- a/syllabus/AREC 615 Class Schedule.xlsx
+++ b/syllabus/AREC 615 Class Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/judebayham/Documents/git_projects/arec-615/syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6120A27-3ED7-114A-BC82-C6F4B36C8A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2485093-CAE1-B44E-85B0-C9D28A4DB70D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36840" yWindow="1120" windowWidth="34560" windowHeight="20320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FA2025" sheetId="6" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
   <si>
     <t>Review</t>
   </si>
@@ -112,15 +112,9 @@
     <t>Linear Programming: formulation and graphical interpretation</t>
   </si>
   <si>
-    <t>LP formulation from data</t>
-  </si>
-  <si>
     <t>LP sensitivity and shadow values</t>
   </si>
   <si>
-    <t>LP duality as economic interpretation</t>
-  </si>
-  <si>
     <t>Presentation/discussion</t>
   </si>
   <si>
@@ -161,6 +155,12 @@
   </si>
   <si>
     <t>McCarl &amp; Spreen Chapter 1</t>
+  </si>
+  <si>
+    <t>Kaiser and Messer Chapter 1</t>
+  </si>
+  <si>
+    <t>LP duality</t>
   </si>
 </sst>
 </file>
@@ -214,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -236,17 +236,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -612,7 +601,7 @@
         <v>10</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E2" s="3"/>
     </row>
@@ -627,12 +616,14 @@
       <c r="C3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="3"/>
+      <c r="D3" s="3" t="s">
+        <v>27</v>
+      </c>
       <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A4" s="2">
-        <f t="shared" ref="A4:A33" si="1">A2+1</f>
+        <f t="shared" ref="A4:A27" si="1">A2+1</f>
         <v>2</v>
       </c>
       <c r="B4" s="4">
@@ -640,7 +631,7 @@
         <v>46266</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -655,7 +646,7 @@
         <v>46268</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="D5" s="3"/>
     </row>
@@ -669,7 +660,7 @@
         <v>46273</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -684,10 +675,10 @@
         <v>46275</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="13" x14ac:dyDescent="0.15">
@@ -700,7 +691,7 @@
         <v>46280</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="7"/>
@@ -715,7 +706,7 @@
         <v>46282</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -725,12 +716,12 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="4">
         <f>B8+7</f>
         <v>46287</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="3"/>
@@ -758,7 +749,7 @@
         <v>46294</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D12" s="3"/>
     </row>
@@ -772,7 +763,7 @@
         <v>46296</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="8"/>
@@ -787,7 +778,7 @@
         <v>46301</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D14" s="7"/>
       <c r="E14" s="3"/>
@@ -802,7 +793,7 @@
         <v>46303</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E15" s="7"/>
     </row>
@@ -816,7 +807,7 @@
         <v>46308</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D16" s="3"/>
     </row>
@@ -830,7 +821,7 @@
         <v>46310</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E17" s="3"/>
     </row>
@@ -844,7 +835,7 @@
         <v>46315</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D18" s="3"/>
     </row>
@@ -871,7 +862,7 @@
         <v>46322</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E20" s="3"/>
     </row>
@@ -885,7 +876,7 @@
         <v>46324</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="7"/>
@@ -900,7 +891,7 @@
         <v>46329</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="7"/>
@@ -915,7 +906,7 @@
         <v>46331</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D23" s="3"/>
     </row>
@@ -929,7 +920,7 @@
         <v>46336</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="14" x14ac:dyDescent="0.15">
@@ -942,7 +933,7 @@
         <v>46338</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D25" s="3"/>
     </row>
@@ -971,48 +962,47 @@
         <v>46345</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
     <row r="28" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A28" s="10"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="11"/>
+      <c r="A28" s="2"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="3"/>
     </row>
     <row r="29" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A29" s="10"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="11"/>
+      <c r="A29" s="2"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="3"/>
     </row>
     <row r="30" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A30" s="10"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="11"/>
+      <c r="A30" s="2"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="3"/>
       <c r="D30" s="3"/>
     </row>
     <row r="31" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A31" s="10"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="11"/>
+      <c r="A31" s="2"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="3"/>
       <c r="D31" s="1"/>
       <c r="E31" s="3"/>
     </row>
     <row r="32" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A32" s="10"/>
-      <c r="B32" s="9"/>
-      <c r="C32" s="12"/>
+      <c r="A32" s="2"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="1"/>
     </row>
     <row r="33" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A33" s="10"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="12"/>
+      <c r="A33" s="2"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="1"/>
     </row>
     <row r="34" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A34" s="13"/>
-      <c r="B34" s="9"/>
-      <c r="C34" s="12"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="1"/>
     </row>
     <row r="35" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="B35" s="4"/>

</xml_diff>

<commit_message>
Update course materials and schedule for Linear Programming module
</commit_message>
<xml_diff>
--- a/syllabus/AREC 615 Class Schedule.xlsx
+++ b/syllabus/AREC 615 Class Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/judebayham/Documents/git_projects/arec-615/syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2485093-CAE1-B44E-85B0-C9D28A4DB70D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3086CE-06E7-EF4A-844C-FD60E72824BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
   <si>
     <t>Review</t>
   </si>
@@ -161,6 +161,12 @@
   </si>
   <si>
     <t>LP duality</t>
+  </si>
+  <si>
+    <t>Kaiser and Messer Chapter 3</t>
+  </si>
+  <si>
+    <t>Baumol - Duality</t>
   </si>
 </sst>
 </file>
@@ -636,7 +642,7 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:5" ht="14" x14ac:dyDescent="0.15">
       <c r="A5" s="2">
         <f t="shared" si="1"/>
         <v>2</v>
@@ -648,9 +654,11 @@
       <c r="C5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="D5" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="14" x14ac:dyDescent="0.15">
       <c r="A6" s="2">
         <f t="shared" si="1"/>
         <v>3</v>
@@ -662,7 +670,9 @@
       <c r="C6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" ht="14" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Add answer key for AREC 615 Linear Programming and update class schedule
- Introduced a new PDF and QMD file containing the answer key for the linear programming problem set, including detailed solutions and checks for independent review.
- Updated the class schedule Excel file for AREC 615 to reflect the latest changes.
</commit_message>
<xml_diff>
--- a/syllabus/AREC 615 Class Schedule.xlsx
+++ b/syllabus/AREC 615 Class Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/judebayham/Documents/git_projects/arec-615/syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3086CE-06E7-EF4A-844C-FD60E72824BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF3F376-C720-5B48-BDA1-513AE3CE21FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
   <si>
     <t>Review</t>
   </si>
@@ -127,24 +127,15 @@
     <t>Midterm 2</t>
   </si>
   <si>
-    <t>Unconstrained and constrained nonlinear optimization + Numerical foundations: roots, diagnostics, and convergence</t>
-  </si>
-  <si>
     <t>Risk, uncertainty, and scenario analysis in static models</t>
   </si>
   <si>
-    <t>Finite-horizon dynamic programming and backward induction</t>
-  </si>
-  <si>
     <t>Infinite-horizon Bellman equation and value function iteration</t>
   </si>
   <si>
     <t>Final</t>
   </si>
   <si>
-    <t>Flex Day</t>
-  </si>
-  <si>
     <t>Stewart &amp; Greenhalgh (1977)</t>
   </si>
   <si>
@@ -167,6 +158,30 @@
   </si>
   <si>
     <t>Baumol - Duality</t>
+  </si>
+  <si>
+    <t>Nonlinear optimization</t>
+  </si>
+  <si>
+    <t>Numeric Methods</t>
+  </si>
+  <si>
+    <t>Build your own</t>
+  </si>
+  <si>
+    <t>Application</t>
+  </si>
+  <si>
+    <t>Intro dynamic programming</t>
+  </si>
+  <si>
+    <t>Discrete time finite horizon: formulation</t>
+  </si>
+  <si>
+    <t>Discrete time finite horizon: solution concepts</t>
+  </si>
+  <si>
+    <t>Schlachtberger et al (2017)</t>
   </si>
 </sst>
 </file>
@@ -569,7 +584,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E982"/>
+  <dimension ref="A1:E986"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="5.1640625" customWidth="1"/>
@@ -607,7 +622,7 @@
         <v>10</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E2" s="3"/>
     </row>
@@ -623,13 +638,13 @@
         <v>11</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A4" s="2">
-        <f t="shared" ref="A4:A27" si="1">A2+1</f>
+        <f t="shared" ref="A4:A29" si="1">A2+1</f>
         <v>2</v>
       </c>
       <c r="B4" s="4">
@@ -637,7 +652,7 @@
         <v>46266</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -655,7 +670,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" x14ac:dyDescent="0.15">
@@ -668,10 +683,10 @@
         <v>46273</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E6" s="3"/>
     </row>
@@ -685,10 +700,10 @@
         <v>46275</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="13" x14ac:dyDescent="0.15">
@@ -706,7 +721,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="7"/>
     </row>
-    <row r="9" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:5" ht="14" x14ac:dyDescent="0.15">
       <c r="A9" s="2">
         <f t="shared" si="1"/>
         <v>4</v>
@@ -716,9 +731,11 @@
         <v>46282</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>35</v>
+      </c>
       <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5" ht="13" x14ac:dyDescent="0.15">
@@ -738,60 +755,60 @@
     </row>
     <row r="11" spans="1:5" ht="14" x14ac:dyDescent="0.15">
       <c r="A11" s="2">
-        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="B11" s="4">
-        <f t="shared" ref="B11" si="5">B10+2</f>
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A12" s="2">
+        <f>A9+1</f>
+        <v>5</v>
+      </c>
+      <c r="B12" s="4">
+        <f t="shared" ref="B12" si="5">B10+2</f>
+        <v>46289</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A13" s="2">
+        <f>A10+1</f>
+        <v>6</v>
+      </c>
+      <c r="B13" s="4">
+        <f>B10+7</f>
+        <v>46294</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+      <c r="A14" s="2">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="B12" s="4">
-        <f>B10+7</f>
-        <v>46294</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A13" s="2">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="B13" s="4">
-        <f t="shared" ref="B13" si="6">B12+2</f>
+      <c r="B14" s="4">
+        <f t="shared" ref="B14" si="6">B13+2</f>
         <v>46296</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="8"/>
-    </row>
-    <row r="14" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A14" s="2">
-        <f t="shared" si="1"/>
-        <v>7</v>
-      </c>
-      <c r="B14" s="4">
-        <f>B12+7</f>
-        <v>46301</v>
-      </c>
       <c r="C14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="3"/>
+        <v>29</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="8"/>
     </row>
     <row r="15" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="2">
@@ -799,258 +816,308 @@
         <v>7</v>
       </c>
       <c r="B15" s="4">
-        <f t="shared" ref="B15" si="7">B14+2</f>
-        <v>46303</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15" s="7"/>
+        <f>B13+7</f>
+        <v>46301</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="7"/>
+      <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="2">
+        <v>7</v>
+      </c>
+      <c r="B16" s="4">
+        <v>46302</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="7"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A17" s="2">
+        <f>A14+1</f>
+        <v>7</v>
+      </c>
+      <c r="B17" s="4">
+        <f t="shared" ref="B17" si="7">B15+2</f>
+        <v>46303</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" s="7"/>
+    </row>
+    <row r="18" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A18" s="2">
+        <f>A15+1</f>
+        <v>8</v>
+      </c>
+      <c r="B18" s="4">
+        <f>B15+7</f>
+        <v>46308</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A19" s="2">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="B16" s="4">
-        <f>B14+7</f>
-        <v>46308</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="3"/>
-    </row>
-    <row r="17" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A17" s="2">
-        <f t="shared" si="1"/>
-        <v>8</v>
-      </c>
-      <c r="B17" s="4">
-        <f t="shared" ref="B17" si="8">B16+2</f>
+      <c r="B19" s="4">
+        <f t="shared" ref="B19" si="8">B18+2</f>
         <v>46310</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A18" s="2">
+      <c r="C19" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A20" s="2">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="B18" s="4">
-        <f>B16+7</f>
+      <c r="B20" s="4">
+        <f>B18+7</f>
         <v>46315</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C20" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="3"/>
-    </row>
-    <row r="19" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A19" s="2">
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+      <c r="A21" s="2">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="B19" s="4">
-        <f t="shared" ref="B19" si="9">B18+2</f>
+      <c r="B21" s="4">
+        <f t="shared" ref="B21" si="9">B20+2</f>
         <v>46317</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C21" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A20" s="2">
+    <row r="22" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+      <c r="A22" s="2">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="B20" s="4">
-        <f>B18+7</f>
-        <v>46322</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="3"/>
-    </row>
-    <row r="21" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A21" s="2">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="B21" s="4">
-        <f t="shared" ref="B21" si="10">B20+2</f>
-        <v>46324</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D21" s="3"/>
-      <c r="E21" s="7"/>
-    </row>
-    <row r="22" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A22" s="2">
-        <f t="shared" si="1"/>
-        <v>11</v>
-      </c>
       <c r="B22" s="4">
         <f>B20+7</f>
-        <v>46329</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" s="3"/>
-      <c r="E22" s="7"/>
+        <v>46322</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="3"/>
     </row>
     <row r="23" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A23" s="2">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B23" s="4">
-        <f t="shared" ref="B23" si="11">B22+2</f>
-        <v>46331</v>
+        <f t="shared" ref="B23" si="10">B22+2</f>
+        <v>46324</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D23" s="3"/>
+      <c r="E23" s="7"/>
     </row>
     <row r="24" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A24" s="2">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B24" s="4">
         <f>B22+7</f>
+        <v>46329</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" s="3"/>
+      <c r="E24" s="7"/>
+    </row>
+    <row r="25" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A25" s="2">
+        <v>11</v>
+      </c>
+      <c r="B25" s="4">
+        <v>46330</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="3"/>
+      <c r="E25" s="7"/>
+    </row>
+    <row r="26" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A26" s="2">
+        <f>A23+1</f>
+        <v>11</v>
+      </c>
+      <c r="B26" s="4">
+        <f t="shared" ref="B26" si="11">B24+2</f>
+        <v>46331</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" s="3"/>
+    </row>
+    <row r="27" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A27" s="2">
+        <f>A24+1</f>
+        <v>12</v>
+      </c>
+      <c r="B27" s="4">
+        <f>B24+7</f>
         <v>46336</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C27" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A25" s="2">
+    <row r="28" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A28" s="2">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="B25" s="4">
-        <f t="shared" ref="B25" si="12">B24+2</f>
+      <c r="B28" s="4">
+        <f t="shared" ref="B28" si="12">B27+2</f>
         <v>46338</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D25" s="3"/>
-    </row>
-    <row r="26" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A26" s="2">
+      <c r="C28" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A29" s="2">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="B26" s="4">
-        <f>B24+7</f>
+      <c r="B29" s="4">
+        <f>B27+7</f>
         <v>46343</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C29" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="3"/>
+      <c r="E29" s="7"/>
+    </row>
+    <row r="30" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+      <c r="A30" s="2">
+        <v>13</v>
+      </c>
+      <c r="B30" s="4">
+        <v>46344</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="7"/>
-    </row>
-    <row r="27" spans="1:5" ht="14" x14ac:dyDescent="0.15">
-      <c r="A27" s="2">
-        <f t="shared" si="1"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="7"/>
+    </row>
+    <row r="31" spans="1:5" ht="14" x14ac:dyDescent="0.15">
+      <c r="A31" s="2">
+        <f>A28+1</f>
         <v>13</v>
       </c>
-      <c r="B27" s="4">
-        <f t="shared" ref="B27" si="13">B26+2</f>
+      <c r="B31" s="4">
+        <f t="shared" ref="B31" si="13">B29+2</f>
         <v>46345</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-    </row>
-    <row r="28" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A28" s="2"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="3"/>
-    </row>
-    <row r="29" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A29" s="2"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="3"/>
-    </row>
-    <row r="30" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A30" s="2"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-    </row>
-    <row r="31" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A31" s="2"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="1"/>
+      <c r="C31" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="3"/>
       <c r="E31" s="3"/>
     </row>
     <row r="32" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A32" s="2"/>
       <c r="B32" s="4"/>
-      <c r="C32" s="1"/>
+      <c r="C32" s="3"/>
     </row>
     <row r="33" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A33" s="2"/>
       <c r="B33" s="4"/>
-      <c r="C33" s="1"/>
+      <c r="C33" s="3"/>
     </row>
     <row r="34" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A34" s="2"/>
       <c r="B34" s="4"/>
-      <c r="C34" s="1"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
     </row>
     <row r="35" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A35" s="2"/>
       <c r="B35" s="4"/>
-      <c r="C35" s="7"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="3"/>
     </row>
     <row r="36" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A36" s="2"/>
       <c r="B36" s="4"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="5"/>
+      <c r="C36" s="1"/>
     </row>
     <row r="37" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A37" s="2"/>
       <c r="B37" s="4"/>
       <c r="C37" s="1"/>
-      <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="B38" s="4"/>
       <c r="C38" s="1"/>
     </row>
     <row r="39" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="C39" s="1"/>
-      <c r="D39" s="7"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="7"/>
     </row>
     <row r="40" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="C40" s="7"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="5"/>
     </row>
     <row r="41" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="B41" s="4"/>
       <c r="C41" s="1"/>
-      <c r="D41" s="7"/>
+      <c r="D41" s="3"/>
     </row>
     <row r="42" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="C42" s="1"/>
     </row>
-    <row r="43" spans="1:5" ht="13" x14ac:dyDescent="0.15"/>
-    <row r="44" spans="1:5" ht="13" x14ac:dyDescent="0.15"/>
-    <row r="45" spans="1:5" ht="13" x14ac:dyDescent="0.15"/>
-    <row r="46" spans="1:5" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="43" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="C43" s="1"/>
+      <c r="D43" s="7"/>
+    </row>
+    <row r="44" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="C44" s="7"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+    </row>
+    <row r="45" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="C45" s="1"/>
+      <c r="D45" s="7"/>
+    </row>
+    <row r="46" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="C46" s="1"/>
+    </row>
     <row r="47" spans="1:5" ht="13" x14ac:dyDescent="0.15"/>
     <row r="48" spans="1:5" ht="13" x14ac:dyDescent="0.15"/>
     <row r="49" ht="13" x14ac:dyDescent="0.15"/>
@@ -1987,8 +2054,12 @@
     <row r="980" ht="13" x14ac:dyDescent="0.15"/>
     <row r="981" ht="13" x14ac:dyDescent="0.15"/>
     <row r="982" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="983" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="984" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="985" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="986" ht="13" x14ac:dyDescent="0.15"/>
   </sheetData>
-  <conditionalFormatting sqref="B2:B37">
+  <conditionalFormatting sqref="B2:B41">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND(ISNUMBER(B2),TRUNC(B2)&lt;TODAY())</formula>
     </cfRule>

</xml_diff>